<commit_message>
TLC: FW-faithful rate control (last-known-good fallback + fast-fail dwell)
Align sim TLC to RS_MNG: search falls back to last known-good rate, failing dwell aborts fast, upscale throttle 200ms, avoid-higher-MCS 1s, drop warm-start MCS clamp. Sim now tracks genie ~99% and lab across all BW. TVA sweep limited to SNR 44..2; RSSI-to-SNR sheet uses Excel formulas + new RSSI-to-SNR Diff column. Update architecture TLC-flow behavior/diagram, README lessons + TVA generator note.
</commit_message>
<xml_diff>
--- a/Results/tva_sim_vs_lab_160mhz.xlsx
+++ b/Results/tva_sim_vs_lab_160mhz.xlsx
@@ -290,12 +290,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$B$2:$B$20</f>
+              <f>'ChartData'!$B$2:$B$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -327,12 +327,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$C$2:$C$20</f>
+              <f>'ChartData'!$C$2:$C$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -364,12 +364,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$D$2:$D$20</f>
+              <f>'ChartData'!$D$2:$D$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -474,12 +474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$E$2:$E$20</f>
+              <f>'ChartData'!$E$2:$E$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$F$2:$F$20</f>
+              <f>'ChartData'!$F$2:$F$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -548,12 +548,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$G$2:$G$20</f>
+              <f>'ChartData'!$G$2:$G$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -658,12 +658,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$H$2:$H$20</f>
+              <f>'ChartData'!$H$2:$H$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -695,12 +695,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$I$2:$I$20</f>
+              <f>'ChartData'!$I$2:$I$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -732,12 +732,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$J$2:$J$20</f>
+              <f>'ChartData'!$J$2:$J$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -842,12 +842,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$K$2:$K$20</f>
+              <f>'ChartData'!$K$2:$K$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -879,12 +879,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$L$2:$L$20</f>
+              <f>'ChartData'!$L$2:$L$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -916,12 +916,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$M$2:$M$20</f>
+              <f>'ChartData'!$M$2:$M$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1026,12 +1026,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$N$2:$N$20</f>
+              <f>'ChartData'!$N$2:$N$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1063,12 +1063,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$O$2:$O$20</f>
+              <f>'ChartData'!$O$2:$O$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1100,12 +1100,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ChartData'!$A$2:$A$20</f>
+              <f>'ChartData'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ChartData'!$P$2:$P$20</f>
+              <f>'ChartData'!$P$2:$P$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1566,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1595,7 +1595,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lab log source: C:\Users\eisack\OneDrive - Intel Corporation\Desktop\Efrat\TLC_Sim\PERModel\RefTVA\tva_11be_160mhz_uhbch69_tx_scd.json    |    RSSI→SNR offset (MCS-knee aligned): 88.9 dB</t>
+          <t>Lab log source: C:\Users\eisack\OneDrive - Intel Corporation\Desktop\Efrat\TLC_Sim\PERModel\RefTVA\tva_11be_160mhz_uhbch69_tx_scd.json    |    RSSI→SNR offset (MCS-knee aligned): 89.0 dB</t>
         </is>
       </c>
     </row>
@@ -1711,10 +1711,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>2065</v>
+        <v>2561</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>13</v>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J3" s="8" t="n">
@@ -1762,10 +1762,10 @@
         </is>
       </c>
       <c r="O3" s="9" t="n">
-        <v>-38.7</v>
+        <v>-44.8</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>2216</v>
+        <v>2422</v>
       </c>
       <c r="Q3" s="9" t="n">
         <v>13</v>
@@ -1794,7 +1794,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>2561</v>
@@ -1845,10 +1845,10 @@
         </is>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-41</v>
+        <v>-47</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>2424</v>
+        <v>2425</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>13</v>
@@ -1877,7 +1877,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>2561</v>
@@ -1928,10 +1928,10 @@
         </is>
       </c>
       <c r="O5" s="9" t="n">
-        <v>-44.8</v>
+        <v>-51</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>2422</v>
+        <v>2343</v>
       </c>
       <c r="Q5" s="9" t="n">
         <v>13</v>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="U5" s="9" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>98%</t>
         </is>
       </c>
     </row>
@@ -1960,13 +1960,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>2561</v>
+        <v>2303</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>160</v>
@@ -1983,19 +1983,19 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>2563</v>
+        <v>2318</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>160</v>
@@ -2011,13 +2011,13 @@
         </is>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-47</v>
+        <v>-54</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>2425</v>
+        <v>2154</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="R6" s="9" t="n">
         <v>160</v>
@@ -2043,13 +2043,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>2561</v>
+        <v>2039</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>160</v>
@@ -2075,10 +2075,10 @@
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>2563</v>
+        <v>2042</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>160</v>
@@ -2094,13 +2094,13 @@
         </is>
       </c>
       <c r="O7" s="9" t="n">
-        <v>-51</v>
+        <v>-57</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>2343</v>
+        <v>1987</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="R7" s="9" t="n">
         <v>160</v>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="U7" s="9" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2126,13 +2126,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2282</v>
+        <v>1830</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>160</v>
@@ -2149,19 +2149,19 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>2318</v>
+        <v>1834</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>160</v>
@@ -2177,13 +2177,13 @@
         </is>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-54</v>
+        <v>-60</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>2154</v>
+        <v>1796</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="R8" s="9" t="n">
         <v>160</v>
@@ -2209,13 +2209,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2016</v>
+        <v>1631</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>160</v>
@@ -2232,19 +2232,19 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>2042</v>
+        <v>1633</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>160</v>
@@ -2260,13 +2260,13 @@
         </is>
       </c>
       <c r="O9" s="9" t="n">
-        <v>-57</v>
+        <v>-63</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>1987</v>
+        <v>1595</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R9" s="9" t="n">
         <v>160</v>
@@ -2292,13 +2292,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1808</v>
+        <v>1460</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>160</v>
@@ -2315,19 +2315,19 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>1834</v>
+        <v>1464</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>160</v>
@@ -2343,13 +2343,13 @@
         </is>
       </c>
       <c r="O10" s="9" t="n">
-        <v>-60</v>
+        <v>-65.90000000000001</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>1796</v>
+        <v>1243</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R10" s="9" t="n">
         <v>160</v>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="U10" s="9" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>93%</t>
         </is>
       </c>
     </row>
@@ -2375,13 +2375,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1608</v>
+        <v>1220</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>160</v>
@@ -2398,19 +2398,19 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>1633</v>
+        <v>1223</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>160</v>
@@ -2426,13 +2426,13 @@
         </is>
       </c>
       <c r="O11" s="9" t="n">
-        <v>-63</v>
+        <v>-69</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>1595</v>
+        <v>1150</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R11" s="9" t="n">
         <v>160</v>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="U11" s="9" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2458,13 +2458,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1438</v>
+        <v>1061</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>160</v>
@@ -2486,14 +2486,14 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>1464</v>
+        <v>1069</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>160</v>
@@ -2509,13 +2509,13 @@
         </is>
       </c>
       <c r="O12" s="9" t="n">
-        <v>-65.90000000000001</v>
+        <v>-72</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>1243</v>
+        <v>854</v>
       </c>
       <c r="Q12" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R12" s="9" t="n">
         <v>160</v>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="U12" s="9" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>94%</t>
         </is>
       </c>
     </row>
@@ -2541,13 +2541,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1156</v>
+        <v>733</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>160</v>
@@ -2564,19 +2564,19 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>1223</v>
+        <v>735</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>160</v>
@@ -2592,13 +2592,13 @@
         </is>
       </c>
       <c r="O13" s="9" t="n">
-        <v>-69</v>
+        <v>-74.7</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>1150</v>
+        <v>708</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="R13" s="9" t="n">
         <v>160</v>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="U13" s="9" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2624,13 +2624,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1039</v>
+        <v>481</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>160</v>
@@ -2652,14 +2652,14 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>1069</v>
+        <v>514</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>160</v>
@@ -2675,13 +2675,13 @@
         </is>
       </c>
       <c r="O14" s="9" t="n">
-        <v>-72</v>
+        <v>-77.09999999999999</v>
       </c>
       <c r="P14" s="9" t="n">
-        <v>854</v>
+        <v>466</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R14" s="9" t="n">
         <v>160</v>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="U14" s="9" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2707,13 +2707,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>679</v>
+        <v>456</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>160</v>
@@ -2730,19 +2730,19 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>735</v>
+        <v>466</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>160</v>
@@ -2758,13 +2758,13 @@
         </is>
       </c>
       <c r="O15" s="9" t="n">
-        <v>-74.7</v>
+        <v>-80</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>708</v>
+        <v>348</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R15" s="9" t="n">
         <v>160</v>
@@ -2790,13 +2790,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>485</v>
+        <v>339</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>160</v>
@@ -2813,19 +2813,19 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>514</v>
+        <v>349</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>160</v>
@@ -2841,13 +2841,13 @@
         </is>
       </c>
       <c r="O16" s="9" t="n">
-        <v>-77.09999999999999</v>
+        <v>-84</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>466</v>
+        <v>115</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R16" s="9" t="n">
         <v>160</v>
@@ -2873,13 +2873,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>440</v>
+        <v>122</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>160</v>
@@ -2896,19 +2896,19 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>466</v>
+        <v>201</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>160</v>
@@ -2920,24 +2920,24 @@
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>0.8µs</t>
+          <t>3.2µs</t>
         </is>
       </c>
       <c r="O17" s="9" t="n">
-        <v>-80</v>
+        <v>-85.2</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>348</v>
+        <v>27</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R17" s="9" t="n">
         <v>160</v>
       </c>
       <c r="S17" s="9" t="inlineStr">
         <is>
-          <t>MIMO</t>
+          <t>SISO</t>
         </is>
       </c>
       <c r="T17" s="9" t="inlineStr">
@@ -2947,301 +2947,9 @@
       </c>
       <c r="U17" s="9" t="inlineStr">
         <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>323</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>160</v>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>0.8µs</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>83%</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="n">
-        <v>349</v>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="L18" s="8" t="n">
-        <v>160</v>
-      </c>
-      <c r="M18" s="8" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>0.8µs</t>
-        </is>
-      </c>
-      <c r="O18" s="9" t="n">
-        <v>-84</v>
-      </c>
-      <c r="P18" s="9" t="n">
-        <v>115</v>
-      </c>
-      <c r="Q18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="9" t="n">
-        <v>160</v>
-      </c>
-      <c r="S18" s="9" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="T18" s="9" t="inlineStr">
-        <is>
-          <t>0.8µs</t>
-        </is>
-      </c>
-      <c r="U18" s="9" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>167</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>160</v>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>69%</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>61%</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="n">
-        <v>201</v>
-      </c>
-      <c r="K19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="8" t="n">
-        <v>160</v>
-      </c>
-      <c r="M19" s="8" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="O19" s="9" t="n">
-        <v>-85.2</v>
-      </c>
-      <c r="P19" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="9" t="n">
-        <v>160</v>
-      </c>
-      <c r="S19" s="9" t="inlineStr">
-        <is>
-          <t>SISO</t>
-        </is>
-      </c>
-      <c r="T19" s="9" t="inlineStr">
-        <is>
-          <t>0.8µs</t>
-        </is>
-      </c>
-      <c r="U19" s="9" t="inlineStr">
-        <is>
           <t>74%</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>77</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>160</v>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>53%</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>58%</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="K20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="8" t="n">
-        <v>160</v>
-      </c>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>SISO</t>
-        </is>
-      </c>
-      <c r="N20" s="8" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="O20" s="9" t="inlineStr"/>
-      <c r="P20" s="9" t="inlineStr"/>
-      <c r="Q20" s="9" t="inlineStr"/>
-      <c r="R20" s="9" t="inlineStr"/>
-      <c r="S20" s="9" t="inlineStr"/>
-      <c r="T20" s="9" t="inlineStr"/>
-      <c r="U20" s="9" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>-4</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>160</v>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>MIMO</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="K21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="8" t="n">
-        <v>160</v>
-      </c>
-      <c r="M21" s="8" t="inlineStr">
-        <is>
-          <t>SISO</t>
-        </is>
-      </c>
-      <c r="N21" s="8" t="inlineStr">
-        <is>
-          <t>3.2µs</t>
-        </is>
-      </c>
-      <c r="O21" s="9" t="inlineStr"/>
-      <c r="P21" s="9" t="inlineStr"/>
-      <c r="Q21" s="9" t="inlineStr"/>
-      <c r="R21" s="9" t="inlineStr"/>
-      <c r="S21" s="9" t="inlineStr"/>
-      <c r="T21" s="9" t="inlineStr"/>
-      <c r="U21" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3257,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3344,16 +3052,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B2" t="n">
-        <v>2065</v>
+        <v>2561</v>
       </c>
       <c r="C2" t="n">
         <v>2563</v>
       </c>
       <c r="D2" t="n">
-        <v>2216</v>
+        <v>2422</v>
       </c>
       <c r="E2" t="n">
         <v>13</v>
@@ -3394,7 +3102,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B3" t="n">
         <v>2561</v>
@@ -3403,7 +3111,7 @@
         <v>2563</v>
       </c>
       <c r="D3" t="n">
-        <v>2424</v>
+        <v>2425</v>
       </c>
       <c r="E3" t="n">
         <v>13</v>
@@ -3444,7 +3152,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B4" t="n">
         <v>2561</v>
@@ -3453,7 +3161,7 @@
         <v>2563</v>
       </c>
       <c r="D4" t="n">
-        <v>2422</v>
+        <v>2343</v>
       </c>
       <c r="E4" t="n">
         <v>13</v>
@@ -3494,25 +3202,25 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B5" t="n">
-        <v>2561</v>
+        <v>2303</v>
       </c>
       <c r="C5" t="n">
-        <v>2563</v>
+        <v>2318</v>
       </c>
       <c r="D5" t="n">
-        <v>2425</v>
+        <v>2154</v>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H5" t="n">
         <v>160</v>
@@ -3544,25 +3252,25 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B6" t="n">
-        <v>2561</v>
+        <v>2039</v>
       </c>
       <c r="C6" t="n">
-        <v>2563</v>
+        <v>2042</v>
       </c>
       <c r="D6" t="n">
-        <v>2343</v>
+        <v>1987</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H6" t="n">
         <v>160</v>
@@ -3594,25 +3302,25 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B7" t="n">
-        <v>2282</v>
+        <v>1830</v>
       </c>
       <c r="C7" t="n">
-        <v>2318</v>
+        <v>1834</v>
       </c>
       <c r="D7" t="n">
-        <v>2154</v>
+        <v>1796</v>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H7" t="n">
         <v>160</v>
@@ -3644,25 +3352,25 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B8" t="n">
-        <v>2016</v>
+        <v>1631</v>
       </c>
       <c r="C8" t="n">
-        <v>2042</v>
+        <v>1633</v>
       </c>
       <c r="D8" t="n">
-        <v>1987</v>
+        <v>1595</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H8" t="n">
         <v>160</v>
@@ -3694,25 +3402,25 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B9" t="n">
-        <v>1808</v>
+        <v>1460</v>
       </c>
       <c r="C9" t="n">
-        <v>1834</v>
+        <v>1464</v>
       </c>
       <c r="D9" t="n">
-        <v>1796</v>
+        <v>1243</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
         <v>160</v>
@@ -3744,25 +3452,25 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B10" t="n">
-        <v>1608</v>
+        <v>1220</v>
       </c>
       <c r="C10" t="n">
-        <v>1633</v>
+        <v>1223</v>
       </c>
       <c r="D10" t="n">
-        <v>1595</v>
+        <v>1150</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H10" t="n">
         <v>160</v>
@@ -3794,25 +3502,25 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B11" t="n">
-        <v>1438</v>
+        <v>1061</v>
       </c>
       <c r="C11" t="n">
-        <v>1464</v>
+        <v>1069</v>
       </c>
       <c r="D11" t="n">
-        <v>1243</v>
+        <v>854</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H11" t="n">
         <v>160</v>
@@ -3844,25 +3552,25 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B12" t="n">
-        <v>1156</v>
+        <v>733</v>
       </c>
       <c r="C12" t="n">
-        <v>1223</v>
+        <v>735</v>
       </c>
       <c r="D12" t="n">
-        <v>1150</v>
+        <v>708</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H12" t="n">
         <v>160</v>
@@ -3894,25 +3602,25 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1039</v>
+        <v>481</v>
       </c>
       <c r="C13" t="n">
-        <v>1069</v>
+        <v>514</v>
       </c>
       <c r="D13" t="n">
-        <v>854</v>
+        <v>466</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
         <v>160</v>
@@ -3944,25 +3652,25 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B14" t="n">
-        <v>679</v>
+        <v>456</v>
       </c>
       <c r="C14" t="n">
-        <v>735</v>
+        <v>466</v>
       </c>
       <c r="D14" t="n">
-        <v>708</v>
+        <v>348</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
         <v>160</v>
@@ -3994,25 +3702,25 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B15" t="n">
-        <v>485</v>
+        <v>339</v>
       </c>
       <c r="C15" t="n">
-        <v>514</v>
+        <v>349</v>
       </c>
       <c r="D15" t="n">
-        <v>466</v>
+        <v>115</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>160</v>
@@ -4044,25 +3752,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B16" t="n">
-        <v>440</v>
+        <v>122</v>
       </c>
       <c r="C16" t="n">
-        <v>466</v>
+        <v>201</v>
       </c>
       <c r="D16" t="n">
-        <v>348</v>
+        <v>27</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>160</v>
@@ -4077,7 +3785,7 @@
         <v>0.8</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8</v>
+        <v>3.2</v>
       </c>
       <c r="M16" t="n">
         <v>0.8</v>
@@ -4089,176 +3797,6 @@
         <v>2</v>
       </c>
       <c r="P16" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B17" t="n">
-        <v>323</v>
-      </c>
-      <c r="C17" t="n">
-        <v>349</v>
-      </c>
-      <c r="D17" t="n">
-        <v>115</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>160</v>
-      </c>
-      <c r="I17" t="n">
-        <v>160</v>
-      </c>
-      <c r="J17" t="n">
-        <v>160</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="N17" t="n">
-        <v>2</v>
-      </c>
-      <c r="O17" t="n">
-        <v>2</v>
-      </c>
-      <c r="P17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" t="n">
-        <v>167</v>
-      </c>
-      <c r="C18" t="n">
-        <v>201</v>
-      </c>
-      <c r="D18" t="n">
-        <v>27</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>160</v>
-      </c>
-      <c r="I18" t="n">
-        <v>160</v>
-      </c>
-      <c r="J18" t="n">
-        <v>160</v>
-      </c>
-      <c r="K18" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L18" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="N18" t="n">
-        <v>2</v>
-      </c>
-      <c r="O18" t="n">
-        <v>2</v>
-      </c>
-      <c r="P18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>-1</v>
-      </c>
-      <c r="B19" t="n">
-        <v>77</v>
-      </c>
-      <c r="C19" t="n">
-        <v>97</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" t="n">
-        <v>160</v>
-      </c>
-      <c r="I19" t="n">
-        <v>160</v>
-      </c>
-      <c r="K19" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L19" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N19" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>-4</v>
-      </c>
-      <c r="B20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C20" t="n">
-        <v>22</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>160</v>
-      </c>
-      <c r="I20" t="n">
-        <v>160</v>
-      </c>
-      <c r="K20" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L20" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N20" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4287,7 +3825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4297,6 +3835,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4309,7 +3848,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Noise Floor = −174 + 10·log10(BW×10^6) + Noise Figure + RSSI implementation Margin ; Estimated RSSI = Noise Floor + required SNR</t>
+          <t>Noise Floor = −174 + 10·log10(BW×10^6) + Noise Figure + RSSI implementation Margin ; Estimated RSSI = Noise Floor + required SNR ; RSSI to SNR Diff = −Noise Floor (add to RSSI to get SNR)</t>
         </is>
       </c>
     </row>
@@ -4347,6 +3886,11 @@
       <c r="G4" s="10" t="inlineStr">
         <is>
           <t>RSSI from model (dBm)</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>RSSI to SNR Diff (dB)</t>
         </is>
       </c>
     </row>
@@ -4360,17 +3904,23 @@
       <c r="C5" s="11" t="n">
         <v>320</v>
       </c>
-      <c r="D5" s="11" t="n">
-        <v>-76.90000000000001</v>
+      <c r="D5" s="11">
+        <f>-174 + 10*LOG10(C5*10^6) + $A$5 + $B$5</f>
+        <v/>
       </c>
       <c r="E5" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="F5" s="11" t="n">
-        <v>-39.9</v>
+      <c r="F5" s="11">
+        <f>D5 + E5</f>
+        <v/>
       </c>
       <c r="G5" s="11" t="n">
         <v>-40</v>
+      </c>
+      <c r="H5" s="11">
+        <f>-D5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -4379,17 +3929,23 @@
       <c r="C6" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="D6" s="11" t="n">
-        <v>-80</v>
+      <c r="D6" s="11">
+        <f>-174 + 10*LOG10(C6*10^6) + $A$5 + $B$5</f>
+        <v/>
       </c>
       <c r="E6" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="F6" s="11" t="n">
-        <v>-43</v>
+      <c r="F6" s="11">
+        <f>D6 + E6</f>
+        <v/>
       </c>
       <c r="G6" s="11" t="n">
         <v>-42</v>
+      </c>
+      <c r="H6" s="11">
+        <f>-D6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -4398,17 +3954,23 @@
       <c r="C7" s="11" t="n">
         <v>80</v>
       </c>
-      <c r="D7" s="11" t="n">
-        <v>-83</v>
+      <c r="D7" s="11">
+        <f>-174 + 10*LOG10(C7*10^6) + $A$5 + $B$5</f>
+        <v/>
       </c>
       <c r="E7" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="F7" s="11" t="n">
-        <v>-46</v>
+      <c r="F7" s="11">
+        <f>D7 + E7</f>
+        <v/>
       </c>
       <c r="G7" s="11" t="n">
         <v>-44.5</v>
+      </c>
+      <c r="H7" s="11">
+        <f>-D7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -4417,17 +3979,23 @@
       <c r="C8" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D8" s="11" t="n">
-        <v>-86</v>
+      <c r="D8" s="11">
+        <f>-174 + 10*LOG10(C8*10^6) + $A$5 + $B$5</f>
+        <v/>
       </c>
       <c r="E8" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="F8" s="11" t="n">
-        <v>-49</v>
+      <c r="F8" s="11">
+        <f>D8 + E8</f>
+        <v/>
       </c>
       <c r="G8" s="11" t="n">
         <v>-47.5</v>
+      </c>
+      <c r="H8" s="11">
+        <f>-D8</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -4436,17 +4004,23 @@
       <c r="C9" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="D9" s="11" t="n">
-        <v>-89</v>
+      <c r="D9" s="11">
+        <f>-174 + 10*LOG10(C9*10^6) + $A$5 + $B$5</f>
+        <v/>
       </c>
       <c r="E9" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>-52</v>
+      <c r="F9" s="11">
+        <f>D9 + E9</f>
+        <v/>
       </c>
       <c r="G9" s="11" t="n">
         <v>-50.5</v>
+      </c>
+      <c r="H9" s="11">
+        <f>-D9</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>